<commit_message>
Bổ sung sheet Thông tin webconfig để cấu hình webconfig mà không cần sửa tay
</commit_message>
<xml_diff>
--- a/ExcelCauHinh/Settup AXE.xlsx
+++ b/ExcelCauHinh/Settup AXE.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\ToolAXE\CauHinhHeThongAXE\IIS\ExcelCauHinh\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBCD0293-CA6C-4442-8ABC-458E718863E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71DEF5B-0D41-4D4C-9007-94E3DD5B49DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cài đặt IIS" sheetId="2" r:id="rId1"/>
     <sheet name="Cài đặt SQL" sheetId="3" r:id="rId2"/>
     <sheet name="Cài đặt service" sheetId="4" r:id="rId3"/>
-    <sheet name="Thông tin AX-DMS" sheetId="1" state="hidden" r:id="rId4"/>
+    <sheet name="Thông tin Webconfig" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="98">
   <si>
     <t>Thông tin chung</t>
   </si>
@@ -216,72 +216,6 @@
     <t>Đường dẫn gốc chứa app Service Export</t>
   </si>
   <si>
-    <t>Script</t>
-  </si>
-  <si>
-    <t>MMDS-ConfigAPI</t>
-  </si>
-  <si>
-    <t>MMDS-File</t>
-  </si>
-  <si>
-    <t>MMDS-Hangfire</t>
-  </si>
-  <si>
-    <t>MMDS-Lgsp</t>
-  </si>
-  <si>
-    <t>MMDS-Log</t>
-  </si>
-  <si>
-    <t>MMDS-Mobile</t>
-  </si>
-  <si>
-    <t>MMDS-Notify</t>
-  </si>
-  <si>
-    <t>MMDS-OCR</t>
-  </si>
-  <si>
-    <t>MMDS-Portal</t>
-  </si>
-  <si>
-    <t>MMDS-Web</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\ConfigAPI"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\File"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Hangfire"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Lgsp"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Log"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Mobile"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Notify"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\OCR"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Portal"</t>
-  </si>
-  <si>
-    <t>"E:\SourceWeb\DAS-MMDS\Web"</t>
-  </si>
-  <si>
-    <t>Tạo Application Pool cho Website/Application</t>
-  </si>
-  <si>
     <t>C:\SourceWeb\CSDL\DB\</t>
   </si>
   <si>
@@ -345,10 +279,49 @@
     <t>C:\SourceWeb\Web\</t>
   </si>
   <si>
-    <t>E:\AXE\DataStorage\Storage</t>
-  </si>
-  <si>
     <t>AXE1_</t>
+  </si>
+  <si>
+    <t>C:\AXE\DataStorage\Storage</t>
+  </si>
+  <si>
+    <t>connectionStrings</t>
+  </si>
+  <si>
+    <t>datasource</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>DB</t>
+  </si>
+  <si>
+    <t>AXE_2026_T05_</t>
+  </si>
+  <si>
+    <t>Thư mục dard</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>C:\SourceWeb\Web\dard</t>
+  </si>
+  <si>
+    <t>Thư mục storage</t>
+  </si>
+  <si>
+    <t>storage web</t>
+  </si>
+  <si>
+    <t>storage service export</t>
+  </si>
+  <si>
+    <t>storage service ocr</t>
+  </si>
+  <si>
+    <t>C:\AXE\DataStorage</t>
   </si>
 </sst>
 </file>
@@ -433,7 +406,7 @@
       <charset val="163"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -461,6 +434,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -570,14 +555,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -637,63 +617,56 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -978,634 +951,641 @@
   <dimension ref="A1:J38"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.88671875" style="11" customWidth="1"/>
-    <col min="3" max="3" width="46" style="25" customWidth="1"/>
-    <col min="4" max="5" width="7.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="147" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="11"/>
-    <col min="10" max="10" width="15" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="34" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.88671875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="46" style="22" customWidth="1"/>
+    <col min="4" max="5" width="7.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="147" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="8"/>
+    <col min="10" max="10" width="15" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="46"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="37"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="17"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="47"/>
+      <c r="B3" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="38"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C4" s="17" t="s">
+      <c r="B4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="47"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="47"/>
+      <c r="B5" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="17" t="s">
+      <c r="B6" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="47"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="17" t="s">
+      <c r="B7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="47"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="48"/>
+      <c r="C8" s="14"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="39"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="20"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="17"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="12"/>
-      <c r="H10" s="13"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="str">
+      <c r="A11" s="18" t="str">
         <f>B3&amp;"-Web"</f>
         <v>AXE-Web</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="12"/>
-      <c r="H11" s="21" t="str">
+      <c r="G11" s="9"/>
+      <c r="H11" s="18" t="str">
         <f>IF(A11="","",$B$8&amp;" add apppool /name:"&amp;A11&amp;" /managedRuntimeVersion:"&amp;B11&amp;" /managedPipelineMode:"&amp;C11&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:AXE-Web /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="17"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="21"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="14"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="13"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="12"/>
-      <c r="H14" s="13"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="str">
+      <c r="A15" s="18" t="str">
         <f>B5&amp;"Web"</f>
         <v>AXE1_Web</v>
       </c>
-      <c r="B15" s="21" t="str">
+      <c r="B15" s="18" t="str">
         <f>$B$4&amp;"dard"</f>
         <v>C:\SourceWeb\Web\dard</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="13">
         <v>8539</v>
       </c>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21" t="str">
+      <c r="E15" s="18"/>
+      <c r="F15" s="18" t="str">
         <f>A11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="G15" s="12"/>
-      <c r="H15" s="21" t="str">
+      <c r="G15" s="9"/>
+      <c r="H15" s="18" t="str">
         <f>IF(A15="","",$B$8&amp;" add site /name:"""&amp;A15&amp;""" /physicalPath:"&amp;B15&amp;" /bindings:"&amp;C15&amp;"/*:"&amp;D15&amp;":"&amp;E15&amp;"" )</f>
         <v>c:\Windows\system32\inetsrv\appcmd add site /name:"AXE1_Web" /physicalPath:C:\SourceWeb\Web\dard /bindings:http/*:8539:</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="21"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="18"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="13"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="13"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="13"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="21" t="str">
+      <c r="B19" s="18" t="str">
         <f t="shared" ref="B19:B24" si="0">$A$15</f>
         <v>AXE1_Web</v>
       </c>
-      <c r="C19" s="17" t="str">
+      <c r="C19" s="14" t="str">
         <f>$B$4&amp;"login"</f>
         <v>C:\SourceWeb\Web\login</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="36" t="s">
+      <c r="E19" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="36"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="21" t="str">
+      <c r="F19" s="46"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="18" t="str">
         <f t="shared" ref="H19:H24" si="1">IF(D19="","",$B$8&amp;" add app  /site.name:"""&amp;B19&amp;""" /path:/"&amp;A19&amp;" /physicalPath:"&amp;C19&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/login /physicalPath:C:\SourceWeb\Web\login</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="21" t="str">
+      <c r="B20" s="18" t="str">
         <f t="shared" si="0"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="C20" s="17" t="str">
+      <c r="C20" s="14" t="str">
         <f>$B$4&amp;"admin"</f>
         <v>C:\SourceWeb\Web\admin</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="36" t="s">
+      <c r="E20" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="36"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="21" t="str">
+      <c r="F20" s="46"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="18" t="str">
         <f t="shared" si="1"/>
         <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/admin /physicalPath:C:\SourceWeb\Web\admin</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="21" t="str">
+      <c r="B21" s="18" t="str">
         <f t="shared" si="0"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="C21" s="17" t="str">
+      <c r="C21" s="14" t="str">
         <f>$B$4&amp;"resumable"</f>
         <v>C:\SourceWeb\Web\resumable</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="36" t="s">
+      <c r="E21" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="36"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="21" t="str">
+      <c r="F21" s="46"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="18" t="str">
         <f t="shared" si="1"/>
         <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/resumable /physicalPath:C:\SourceWeb\Web\resumable</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="21" t="str">
+      <c r="B22" s="18" t="str">
         <f t="shared" si="0"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="C22" s="17" t="str">
+      <c r="C22" s="14" t="str">
         <f>$B$4&amp;"uploader"</f>
         <v>C:\SourceWeb\Web\uploader</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="36" t="s">
+      <c r="E22" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="36"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="21" t="str">
+      <c r="F22" s="46"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="18" t="str">
         <f t="shared" si="1"/>
         <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/uploader /physicalPath:C:\SourceWeb\Web\uploader</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="21" t="str">
+      <c r="B23" s="18" t="str">
         <f t="shared" si="0"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="C23" s="17" t="str">
+      <c r="C23" s="14" t="str">
         <f>$B$7</f>
-        <v>E:\AXE\DataStorage\Storage</v>
-      </c>
-      <c r="D23" s="22" t="s">
+        <v>C:\AXE\DataStorage\Storage</v>
+      </c>
+      <c r="D23" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="36" t="s">
+      <c r="E23" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="36"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="21" t="str">
+      <c r="F23" s="46"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="18" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/storage /physicalPath:E:\AXE\DataStorage\Storage</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/storage /physicalPath:C:\AXE\DataStorage\Storage</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="21" t="str">
+      <c r="B24" s="18" t="str">
         <f t="shared" si="0"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="C24" s="17" t="str">
+      <c r="C24" s="14" t="str">
         <f>$B$4&amp;"sohoa"</f>
         <v>C:\SourceWeb\Web\sohoa</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="36" t="s">
+      <c r="E24" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="36"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="21" t="str">
+      <c r="F24" s="46"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="18" t="str">
         <f t="shared" si="1"/>
         <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE1_Web" /path:/doc /physicalPath:C:\SourceWeb\Web\sohoa</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="21"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="18"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="H26" s="13"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H27" s="13"/>
+      <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="21" t="str">
+      <c r="A28" s="18" t="str">
         <f>$A$15</f>
         <v>AXE1_Web</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="17" t="str">
+      <c r="B28" s="18"/>
+      <c r="C28" s="14" t="str">
         <f>$A$11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="H28" s="21" t="str">
+      <c r="H28" s="18" t="str">
         <f>IF(C28="","",$B$8&amp;" set app "&amp;A28&amp;"/  /"&amp;"applicationPool:"&amp;C28&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="H29" s="21"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="21"/>
+      <c r="H29" s="18"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="45"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="H30" s="21"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="36"/>
+      <c r="F30" s="36"/>
+      <c r="H30" s="18"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="C31" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="50" t="s">
+      <c r="D31" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="H31" s="21"/>
+      <c r="E31" s="41"/>
+      <c r="F31" s="41"/>
+      <c r="H31" s="18"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="str">
+      <c r="A32" s="18" t="str">
         <f>$A$15</f>
         <v>AXE1_Web</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="17" t="str">
+      <c r="C32" s="14" t="str">
         <f>$A$11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
-      <c r="H32" s="21" t="str">
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="H32" s="18" t="str">
         <f>IF(C32="","",$B$8&amp;" set app "&amp;A32&amp;"/"&amp;B32&amp;"  /"&amp;"applicationPool:"&amp;C32&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/login  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="21" t="str">
+      <c r="A33" s="18" t="str">
         <f t="shared" ref="A33:A37" si="2">$A$15</f>
         <v>AXE1_Web</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="17" t="str">
+      <c r="C33" s="14" t="str">
         <f t="shared" ref="C33:C37" si="3">$A$11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="H33" s="21" t="str">
+      <c r="D33" s="40"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
+      <c r="H33" s="18" t="str">
         <f>IF(C33="","",$B$8&amp;" set app "&amp;A33&amp;"/"&amp;B33&amp;"  /"&amp;"applicationPool:"&amp;C33&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/admin  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="21" t="str">
+      <c r="A34" s="18" t="str">
         <f t="shared" si="2"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="17" t="str">
+      <c r="C34" s="14" t="str">
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="H34" s="21" t="str">
+      <c r="D34" s="40"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="H34" s="18" t="str">
         <f>IF(C34="","",$B$8&amp;" set app "&amp;A34&amp;"/"&amp;B34&amp;"  /"&amp;"applicationPool:"&amp;C34&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/resumable  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="str">
+      <c r="A35" s="18" t="str">
         <f t="shared" si="2"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="17" t="str">
+      <c r="C35" s="14" t="str">
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="H35" s="21" t="str">
+      <c r="D35" s="40"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="40"/>
+      <c r="H35" s="18" t="str">
         <f>IF(C35="","",$B$8&amp;" set app "&amp;A35&amp;"/"&amp;B35&amp;"  /"&amp;"applicationPool:"&amp;C35&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/uploader  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="str">
+      <c r="A36" s="18" t="str">
         <f t="shared" si="2"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="17" t="str">
+      <c r="C36" s="14" t="str">
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
-      <c r="H36" s="21" t="str">
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
+      <c r="H36" s="18" t="str">
         <f>IF(C36="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A36&amp;"/"&amp;B36&amp;"  /"&amp;"applicationPool:"&amp;C36&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/storage  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="21" t="str">
+      <c r="A37" s="18" t="str">
         <f t="shared" si="2"/>
         <v>AXE1_Web</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="17" t="str">
+      <c r="C37" s="14" t="str">
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D37" s="42"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="44"/>
-      <c r="H37" s="21" t="str">
+      <c r="D37" s="33"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="35"/>
+      <c r="H37" s="18" t="str">
         <f t="shared" ref="H37:H38" si="4">IF(C37="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A37&amp;"/"&amp;B37&amp;"  /"&amp;"applicationPool:"&amp;C37&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/doc  /applicationPool:AXE-Web</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="21"/>
-      <c r="B38" s="21"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="44"/>
-      <c r="H38" s="21" t="str">
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="35"/>
+      <c r="H38" s="18" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="H1:J1"/>
@@ -1622,13 +1602,6 @@
     <mergeCell ref="D35:F35"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K427:K1048576 G26:G426 K1:K25 B18 G9:G10" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1658,208 +1631,208 @@
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="255.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="34.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="255.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="46"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="21"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="47"/>
+      <c r="B3" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="18"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="21"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="47"/>
+      <c r="B4" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="18"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="38"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="47"/>
+      <c r="C5" s="18"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="38"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="29">
         <v>123456</v>
       </c>
-      <c r="C6" s="21"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="47"/>
+      <c r="C6" s="18"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="38"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="20"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="18">
         <v>123456</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="21" t="str">
+      <c r="C9" s="18"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="18" t="str">
         <f>IF(D2="","","CREATE LOGIN "&amp;A9&amp;" WITH PASSWORD = '"&amp;B9&amp;"', CHECK_POLICY = OFF,           CHECK_EXPIRATION = OFF;")</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="21"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="18"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="21" t="str">
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="18" t="str">
         <f>"DECLARE @DataLogicalName NVARCHAR(128);DECLARE @LogLogicalName NVARCHAR(128);"</f>
         <v>DECLARE @DataLogicalName NVARCHAR(128);DECLARE @LogLogicalName NVARCHAR(128);</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="33"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="21" t="s">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="18" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="10"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="10"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" s="27" t="str">
+      <c r="A15" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="24" t="str">
         <f>B3&amp;A15</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_ACC.bak</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15" s="30" t="str">
+      <c r="C15" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="27" t="str">
         <f>$B$4&amp;$C15&amp;".mdf"</f>
         <v>D:\T05\Database\AXE_2026_T05_ACC.mdf</v>
       </c>
-      <c r="E15" s="30" t="str">
+      <c r="E15" s="27" t="str">
         <f>$B$4&amp;$C15&amp;".ldf"</f>
         <v>D:\T05\Database\AXE_2026_T05_ACC.ldf</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="35" t="str">
+      <c r="F15" s="9"/>
+      <c r="G15" s="32" t="str">
         <f>"INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN,"&amp;" BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)"&amp;"
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''"&amp;B15&amp;"''');"&amp;"
 UPDATE #FileList SET PhysicalPath = '"&amp;B15&amp;"' WHERE PhysicalPath IS NULL;"&amp;"
@@ -1884,26 +1857,26 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="B16" s="30" t="str">
+      <c r="A16" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="27" t="str">
         <f>B3&amp;A16</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_CLOUD.bak</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>92</v>
-      </c>
-      <c r="D16" s="30" t="str">
+      <c r="C16" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="27" t="str">
         <f>$B$4&amp;$C16&amp;".mdf"</f>
         <v>D:\T05\Database\AXE_2026_T05_CLOUD.mdf</v>
       </c>
-      <c r="E16" s="30" t="str">
+      <c r="E16" s="27" t="str">
         <f>$B$4&amp;$C16&amp;".ldf"</f>
         <v>D:\T05\Database\AXE_2026_T05_CLOUD.ldf</v>
       </c>
-      <c r="F16" s="12"/>
-      <c r="G16" s="35" t="str">
+      <c r="F16" s="9"/>
+      <c r="G16" s="32" t="str">
         <f>"INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN,"&amp;" BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)"&amp;"
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''"&amp;B16&amp;"''');"&amp;"
 UPDATE #FileList SET PhysicalPath = '"&amp;B16&amp;"' WHERE PhysicalPath IS NULL;"&amp;"
@@ -1928,26 +1901,26 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" s="30" t="str">
+      <c r="A17" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="27" t="str">
         <f>B3&amp;A17</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_CNF.bak</v>
       </c>
-      <c r="C17" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="D17" s="30" t="str">
+      <c r="C17" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="27" t="str">
         <f t="shared" ref="D17:D20" si="0">$B$4&amp;$C17&amp;".mdf"</f>
         <v>D:\T05\Database\AXE_2026_T05_CNF.mdf</v>
       </c>
-      <c r="E17" s="30" t="str">
+      <c r="E17" s="27" t="str">
         <f t="shared" ref="E17:E20" si="1">$B$4&amp;$C17&amp;".ldf"</f>
         <v>D:\T05\Database\AXE_2026_T05_CNF.ldf</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="35" t="str">
+      <c r="F17" s="9"/>
+      <c r="G17" s="32" t="str">
         <f t="shared" ref="G17:G20" si="2">"INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN,"&amp;" BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)"&amp;"
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''"&amp;B17&amp;"''');"&amp;"
 UPDATE #FileList SET PhysicalPath = '"&amp;B17&amp;"' WHERE PhysicalPath IS NULL;"&amp;"
@@ -1972,26 +1945,26 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" s="30" t="str">
+      <c r="A18" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="27" t="str">
         <f>B3&amp;A18</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_LOG.bak</v>
       </c>
-      <c r="C18" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="D18" s="30" t="str">
+      <c r="C18" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="27" t="str">
         <f t="shared" si="0"/>
         <v>D:\T05\Database\AXE_2026_T05_LOG.mdf</v>
       </c>
-      <c r="E18" s="30" t="str">
+      <c r="E18" s="27" t="str">
         <f t="shared" si="1"/>
         <v>D:\T05\Database\AXE_2026_T05_LOG.ldf</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="35" t="str">
+      <c r="F18" s="9"/>
+      <c r="G18" s="32" t="str">
         <f t="shared" si="2"/>
         <v>INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN, BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''C:\SourceWeb\CSDL\DB\AXE_2026_T05_LOG.bak''');
@@ -2006,26 +1979,26 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="30" t="str">
+      <c r="A19" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" s="27" t="str">
         <f>B3&amp;A19</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_MSG.bak</v>
       </c>
-      <c r="C19" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="D19" s="30" t="str">
+      <c r="C19" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="27" t="str">
         <f t="shared" si="0"/>
         <v>D:\T05\Database\AXE_2026_T05_MSG.mdf</v>
       </c>
-      <c r="E19" s="30" t="str">
+      <c r="E19" s="27" t="str">
         <f t="shared" si="1"/>
         <v>D:\T05\Database\AXE_2026_T05_MSG.ldf</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="35" t="str">
+      <c r="F19" s="9"/>
+      <c r="G19" s="32" t="str">
         <f t="shared" si="2"/>
         <v>INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN, BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''C:\SourceWeb\CSDL\DB\AXE_2026_T05_MSG.bak''');
@@ -2040,26 +2013,26 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="30" t="str">
+      <c r="A20" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="27" t="str">
         <f>B3&amp;A20</f>
         <v>C:\SourceWeb\CSDL\DB\AXE_2026_T05_STG.bak</v>
       </c>
-      <c r="C20" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="D20" s="30" t="str">
+      <c r="C20" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="27" t="str">
         <f t="shared" si="0"/>
         <v>D:\T05\Database\AXE_2026_T05_STG.mdf</v>
       </c>
-      <c r="E20" s="30" t="str">
+      <c r="E20" s="27" t="str">
         <f t="shared" si="1"/>
         <v>D:\T05\Database\AXE_2026_T05_STG.ldf</v>
       </c>
-      <c r="F20" s="12"/>
-      <c r="G20" s="35" t="str">
+      <c r="F20" s="9"/>
+      <c r="G20" s="32" t="str">
         <f t="shared" si="2"/>
         <v>INSERT INTO #FileList (LogicalName, PhysicalName, Type, FileGroupName, Size, MaxSize, FileId, CreateLSN, DropLSN, UniqueId, ReadOnlyLSN, ReadWriteLSN, BackupSizeInBytes, SourceBlockSize, FileGroupId, LogGroupGUID, DifferentialBaseLSN, DifferentialBaseGUID, IsReadOnly, IsPresent, TDEThumbprint, SnapshotUrl)
 EXEC ('RESTORE FILELISTONLY FROM DISK = ''C:\SourceWeb\CSDL\DB\AXE_2026_T05_STG.bak''');
@@ -2117,58 +2090,58 @@
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="9"/>
+      <c r="B2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="6"/>
       <c r="D2" t="str">
         <f>"sc create "&amp;B2&amp;" binPath= """&amp;B3&amp;""" start= auto"</f>
         <v>sc create ServiceOCR1 binPath= "C:\SourceWeb\SERVICE\ServiceOCR\DocProService.exe" start= auto</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C3" s="9"/>
+      <c r="B3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="6"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="9"/>
+      <c r="B4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="6"/>
       <c r="D4" t="str">
         <f>"sc create "&amp;B4&amp;" binPath= """&amp;B5&amp;""" start= auto"</f>
         <v>sc create ServiceExport binPath= "C:\SourceWeb\SERVICE\ServiceExport\DocProService.exe" start= auto</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="9"/>
+      <c r="B5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="6"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="9"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2176,690 +2149,136 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1500CE9D-A3F9-42DA-B277-1145613BDD26}">
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="135.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5546875" customWidth="1"/>
+    <col min="2" max="2" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="54" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="2" t="str">
-        <f>IF(A4="","","c:\Windows\system32\inetsrv\appcmd add apppool /name:"&amp;A4&amp;" /managedRuntimeVersion:"&amp;B4&amp;" /managedPipelineMode:"&amp;C4&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-ConfigAPI /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="2" t="str">
-        <f t="shared" ref="H5:H13" si="0">IF(A5="","","c:\Windows\system32\inetsrv\appcmd add apppool /name:"&amp;A5&amp;" /managedRuntimeVersion:"&amp;B5&amp;" /managedPipelineMode:"&amp;C5&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-File /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Hangfire /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Lgsp /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Log /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Mobile /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Notify /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-OCR /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Portal /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:MMDS-Web /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="2" t="str">
-        <f>IF(A14="","","%systemroot%\system32\inetsrv\appcmd add apppool /name:"&amp;A14&amp;" /managedRuntimeVersion:"&amp;B14&amp;" /managedPipelineMode:"&amp;C14&amp;"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="53"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="2">
-        <v>8090</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="2" t="str">
-        <f>IF(A17="","","c:\Windows\system32\inetsrv\appcmd add site /name:"&amp;A17&amp;" /physicalPath:"&amp;B17&amp;" /bindings:"&amp;C17&amp;"/*:"&amp;D17&amp;":"&amp;E17&amp;"" )</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-ConfigAPI /physicalPath:"E:\SourceWeb\DAS-MMDS\ConfigAPI" /bindings:http/*:8090:</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="2">
-        <v>8089</v>
-      </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G18" s="4"/>
-      <c r="H18" s="2" t="str">
-        <f t="shared" ref="H18:H26" si="1">IF(A18="","","c:\Windows\system32\inetsrv\appcmd add site /name:"&amp;A18&amp;" /physicalPath:"&amp;B18&amp;" /bindings:"&amp;C18&amp;"/*:"&amp;D18&amp;":"&amp;E18&amp;"" )</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-File /physicalPath:"E:\SourceWeb\DAS-MMDS\File" /bindings:http/*:8089:</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="2">
-        <v>8088</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Hangfire /physicalPath:"E:\SourceWeb\DAS-MMDS\Hangfire" /bindings:http/*:8088:</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D20" s="2">
-        <v>8087</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Lgsp /physicalPath:"E:\SourceWeb\DAS-MMDS\Lgsp" /bindings:http/*:8087:</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D21" s="2">
-        <v>8086</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Log /physicalPath:"E:\SourceWeb\DAS-MMDS\Log" /bindings:http/*:8086:</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="2">
-        <v>8085</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Mobile /physicalPath:"E:\SourceWeb\DAS-MMDS\Mobile" /bindings:http/*:8085:</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="2">
-        <v>8084</v>
-      </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Notify /physicalPath:"E:\SourceWeb\DAS-MMDS\Notify" /bindings:http/*:8084:</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="2">
-        <v>8083</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-OCR /physicalPath:"E:\SourceWeb\DAS-MMDS\OCR" /bindings:http/*:8083:</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="2">
-        <v>8082</v>
-      </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Portal /physicalPath:"E:\SourceWeb\DAS-MMDS\Portal" /bindings:http/*:8082:</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="2">
-        <v>8081</v>
-      </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:MMDS-Web /physicalPath:"E:\SourceWeb\DAS-MMDS\Web" /bindings:http/*:8081:</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="2" t="str">
-        <f>IF(A27="","","%systemroot%\system32\inetsrv\appcmd add app  /site.name:"&amp;B27&amp;" /path:/"&amp;A27&amp;" /physicalPath:"&amp;C27&amp;"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="54" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="54"/>
-      <c r="C28" s="54"/>
-      <c r="H28" s="1"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H29" s="1"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H30" s="2" t="str">
-        <f>IF(C30="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A30&amp;"/  /"&amp;"applicationPool:"&amp;C30&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-ConfigAPI/  /applicationPool:MMDS-ConfigAPI</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H31" s="2" t="str">
-        <f t="shared" ref="H31:H39" si="2">IF(C31="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A31&amp;"/  /"&amp;"applicationPool:"&amp;C31&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-File/  /applicationPool:MMDS-File</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H32" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Hangfire/  /applicationPool:MMDS-Hangfire</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H33" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Lgsp/  /applicationPool:MMDS-Lgsp</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H34" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Log/  /applicationPool:MMDS-Log</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H35" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Mobile/  /applicationPool:MMDS-Mobile</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="H36" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Notify/  /applicationPool:MMDS-Notify</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H37" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-OCR/  /applicationPool:MMDS-OCR</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="H38" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Portal/  /applicationPool:MMDS-Portal</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H39" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>c:\Windows\system32\inetsrv\appcmd set app MMDS-Web/  /applicationPool:MMDS-Web</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="48" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="50" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="str">
+        <f>"&lt;add name=""accconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"ACC;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="accconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_ACC;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="str">
+        <f>"&lt;add name=""cnfconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"CNF;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="cnfconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_CNF;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="str">
+        <f>"&lt;add name=""stgconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"STG;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="stgconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_STG;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="str">
+        <f>"&lt;add name=""logconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"LOG;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="logconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_LOG;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="str">
+        <f>"&lt;add name=""msgconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"MSG;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="msgconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_MSG;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="str">
+        <f>"&lt;add name=""ctlconnectionstring"" connectionString=""data source="&amp;$B$1&amp;";initial catalog="&amp;$B$2&amp;"CLOUD;integrated security=false;user id=dev;password=123456"" providerName=""system.data.sqlclient"" /&gt;"</f>
+        <v>&lt;add name="ctlconnectionstring" connectionString="data source=.;initial catalog=AXE_2026_T05_CLOUD;integrated security=false;user id=dev;password=123456" providerName="system.data.sqlclient" /&gt;</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="51" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="str">
+        <f>"&lt;add key=""StgBase"" value="""&amp;$B$11&amp;""" /&gt;"</f>
+        <v>&lt;add key="StgBase" value="C:\SourceWeb\Web\dard" /&gt;</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="51" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="49" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="52" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" t="str">
+        <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;""" /&gt;"</f>
+        <v>&lt;add key="StgDir" value="C:\AXE\DataStorage" /&gt;</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="52" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" t="str">
+        <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;"\Storage\Files"" /&gt;"</f>
+        <v>&lt;add key="StgDir" value="C:\AXE\DataStorage\Storage\Files" /&gt;</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="52" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="str">
+        <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;""" /&gt;"</f>
+        <v>&lt;add key="StgDir" value="C:\AXE\DataStorage" /&gt;</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1463:C1048576 C3:C14" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>"Integrated,Classic"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G439:G1048576 C15:C26 G15:G27" xr:uid="{00000000-0002-0000-0300-000001000000}">
-      <formula1>"http,https"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 H439:H1048576 M439:M1048576 H15:H16 E4:E14 H3 H28:H29 M1:M27 I28:I438" xr:uid="{00000000-0002-0000-0300-000002000000}">
-      <formula1>$A$4:$A$14</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K439:K1048576 G2:G3 B27 K1:K27 G28:G438" xr:uid="{00000000-0002-0000-0300-000003000000}">
-      <formula1>$E$4:$E$14</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
-    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010097FE9C0C8E574444875F1CBBF8414DDA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c7e0992f45b677c2156c5ab52d17057f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="97d068c0-5bfb-413b-9996-819e39fdf128" xmlns:ns3="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f06a3ea3329379ac3c4a4f5da7fed49" ns2:_="" ns3:_="">
     <xsd:import namespace="97d068c0-5bfb-413b-9996-819e39fdf128"/>
@@ -3094,26 +2513,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
-    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E3A15DF-6B1B-40AC-992D-CB264AF46DCF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3130,4 +2551,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
+    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cập nhật tool service có thể tạo nhiều service cùng lúc, và phân biệt loại service ở cột Ghi chú
</commit_message>
<xml_diff>
--- a/ExcelCauHinh/Settup AXE.xlsx
+++ b/ExcelCauHinh/Settup AXE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\ToolAXE\CauHinhHeThongAXE\ExcelCauHinh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71DEF5B-0D41-4D4C-9007-94E3DD5B49DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D13DB2F-B25B-425E-A550-C8AA194D0793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cài đặt IIS" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
   <si>
     <t>Thông tin chung</t>
   </si>
@@ -264,9 +264,6 @@
     <t>C:\SourceWeb\SERVICE\ServiceOCR\DocProService.exe</t>
   </si>
   <si>
-    <t>ServiceOCR1</t>
-  </si>
-  <si>
     <t>D:\T05\Database\</t>
   </si>
   <si>
@@ -322,6 +319,21 @@
   </si>
   <si>
     <t>C:\AXE\DataStorage</t>
+  </si>
+  <si>
+    <t>OCR</t>
+  </si>
+  <si>
+    <t>EXPORT</t>
+  </si>
+  <si>
+    <t>ServiceOCR11</t>
+  </si>
+  <si>
+    <t>&lt;add key="AddressOCR" value="11111" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;add key="AXDESHost" value="2222" /&gt;</t>
   </si>
 </sst>
 </file>
@@ -555,7 +567,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -617,56 +629,55 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -967,15 +978,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
       <c r="G1" s="9"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -988,68 +999,68 @@
         <v>3</v>
       </c>
       <c r="G2" s="9"/>
-      <c r="H2" s="37"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" s="14"/>
       <c r="G3" s="9"/>
-      <c r="H3" s="38"/>
+      <c r="H3" s="48"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="9"/>
-      <c r="H4" s="38"/>
+      <c r="H4" s="48"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C5" s="14"/>
       <c r="G5" s="9"/>
-      <c r="H5" s="38"/>
+      <c r="H5" s="48"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="9"/>
-      <c r="H6" s="38"/>
+      <c r="H6" s="48"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
       <c r="G7" s="9"/>
-      <c r="H7" s="38"/>
+      <c r="H7" s="48"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
@@ -1060,17 +1071,17 @@
       </c>
       <c r="C8" s="14"/>
       <c r="G8" s="9"/>
-      <c r="H8" s="39"/>
+      <c r="H8" s="49"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="45"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
       <c r="G9" s="9"/>
       <c r="H9" s="17"/>
     </row>
@@ -1112,14 +1123,14 @@
       <c r="H12" s="18"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="47"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="42"/>
       <c r="G13" s="9"/>
       <c r="H13" s="10"/>
     </row>
@@ -1182,14 +1193,14 @@
       <c r="H16" s="18"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
       <c r="G17" s="9"/>
       <c r="H17" s="10"/>
     </row>
@@ -1228,10 +1239,10 @@
       <c r="D19" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="46" t="s">
+      <c r="E19" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="46"/>
+      <c r="F19" s="37"/>
       <c r="G19" s="9"/>
       <c r="H19" s="18" t="str">
         <f t="shared" ref="H19:H24" si="1">IF(D19="","",$B$8&amp;" add app  /site.name:"""&amp;B19&amp;""" /path:/"&amp;A19&amp;" /physicalPath:"&amp;C19&amp;"")</f>
@@ -1253,10 +1264,10 @@
       <c r="D20" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="46" t="s">
+      <c r="E20" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="46"/>
+      <c r="F20" s="37"/>
       <c r="G20" s="9"/>
       <c r="H20" s="18" t="str">
         <f t="shared" si="1"/>
@@ -1278,10 +1289,10 @@
       <c r="D21" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="46" t="s">
+      <c r="E21" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="46"/>
+      <c r="F21" s="37"/>
       <c r="G21" s="9"/>
       <c r="H21" s="18" t="str">
         <f t="shared" si="1"/>
@@ -1303,10 +1314,10 @@
       <c r="D22" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="46" t="s">
+      <c r="E22" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="46"/>
+      <c r="F22" s="37"/>
       <c r="G22" s="9"/>
       <c r="H22" s="18" t="str">
         <f t="shared" si="1"/>
@@ -1328,10 +1339,10 @@
       <c r="D23" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="46"/>
+      <c r="F23" s="37"/>
       <c r="G23" s="9"/>
       <c r="H23" s="18" t="str">
         <f t="shared" si="1"/>
@@ -1353,10 +1364,10 @@
       <c r="D24" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="46" t="s">
+      <c r="E24" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="46"/>
+      <c r="F24" s="37"/>
       <c r="G24" s="9"/>
       <c r="H24" s="18" t="str">
         <f t="shared" si="1"/>
@@ -1368,20 +1379,20 @@
       <c r="B25" s="18"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
       <c r="G25" s="9"/>
       <c r="H25" s="18"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1418,14 +1429,14 @@
       <c r="H29" s="18"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="36"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
       <c r="H30" s="18"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1438,11 +1449,11 @@
       <c r="C31" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="41"/>
-      <c r="F31" s="41"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="51"/>
       <c r="H31" s="18"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1457,9 +1468,9 @@
         <f>$A$11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
       <c r="H32" s="18" t="str">
         <f>IF(C32="","",$B$8&amp;" set app "&amp;A32&amp;"/"&amp;B32&amp;"  /"&amp;"applicationPool:"&amp;C32&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/login  /applicationPool:AXE-Web</v>
@@ -1477,9 +1488,9 @@
         <f t="shared" ref="C33:C37" si="3">$A$11</f>
         <v>AXE-Web</v>
       </c>
-      <c r="D33" s="40"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
+      <c r="D33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="50"/>
       <c r="H33" s="18" t="str">
         <f>IF(C33="","",$B$8&amp;" set app "&amp;A33&amp;"/"&amp;B33&amp;"  /"&amp;"applicationPool:"&amp;C33&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/admin  /applicationPool:AXE-Web</v>
@@ -1497,9 +1508,9 @@
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D34" s="40"/>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
       <c r="H34" s="18" t="str">
         <f>IF(C34="","",$B$8&amp;" set app "&amp;A34&amp;"/"&amp;B34&amp;"  /"&amp;"applicationPool:"&amp;C34&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/resumable  /applicationPool:AXE-Web</v>
@@ -1517,9 +1528,9 @@
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D35" s="40"/>
-      <c r="E35" s="40"/>
-      <c r="F35" s="40"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="50"/>
       <c r="H35" s="18" t="str">
         <f>IF(C35="","",$B$8&amp;" set app "&amp;A35&amp;"/"&amp;B35&amp;"  /"&amp;"applicationPool:"&amp;C35&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/uploader  /applicationPool:AXE-Web</v>
@@ -1537,9 +1548,9 @@
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D36" s="40"/>
-      <c r="E36" s="40"/>
-      <c r="F36" s="40"/>
+      <c r="D36" s="50"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="50"/>
       <c r="H36" s="18" t="str">
         <f>IF(C36="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A36&amp;"/"&amp;B36&amp;"  /"&amp;"applicationPool:"&amp;C36&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/storage  /applicationPool:AXE-Web</v>
@@ -1557,9 +1568,9 @@
         <f t="shared" si="3"/>
         <v>AXE-Web</v>
       </c>
-      <c r="D37" s="33"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="35"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="44"/>
+      <c r="F37" s="45"/>
       <c r="H37" s="18" t="str">
         <f t="shared" ref="H37:H38" si="4">IF(C37="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A37&amp;"/"&amp;B37&amp;"  /"&amp;"applicationPool:"&amp;C37&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE1_Web/doc  /applicationPool:AXE-Web</v>
@@ -1569,9 +1580,9 @@
       <c r="A38" s="18"/>
       <c r="B38" s="18"/>
       <c r="C38" s="14"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="35"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="44"/>
+      <c r="F38" s="45"/>
       <c r="H38" s="18" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -1579,13 +1590,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E23:F23"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="H1:J1"/>
@@ -1602,6 +1606,13 @@
     <mergeCell ref="D35:F35"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K427:K1048576 G26:G426 K1:K25 B18 G9:G10" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1645,11 +1656,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
       <c r="D1" s="23"/>
       <c r="E1" s="23"/>
       <c r="F1" s="9"/>
@@ -1668,7 +1679,7 @@
       <c r="D2" s="28"/>
       <c r="E2" s="28"/>
       <c r="F2" s="9"/>
-      <c r="G2" s="37"/>
+      <c r="G2" s="47"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -1679,18 +1690,18 @@
       </c>
       <c r="C3" s="18"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="38"/>
+      <c r="G3" s="48"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>45</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="18"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="38"/>
+      <c r="G4" s="48"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
@@ -1701,7 +1712,7 @@
       </c>
       <c r="C5" s="18"/>
       <c r="F5" s="9"/>
-      <c r="G5" s="38"/>
+      <c r="G5" s="48"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
@@ -1712,14 +1723,14 @@
       </c>
       <c r="C6" s="18"/>
       <c r="F6" s="9"/>
-      <c r="G6" s="38"/>
+      <c r="G6" s="48"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
       <c r="D7" s="23"/>
       <c r="E7" s="23"/>
       <c r="F7" s="9"/>
@@ -1753,11 +1764,11 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
       <c r="D10" s="23"/>
       <c r="E10" s="23"/>
       <c r="F10" s="9"/>
@@ -1783,11 +1794,11 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="41"/>
       <c r="D13" s="23"/>
       <c r="E13" s="23"/>
       <c r="F13" s="9"/>
@@ -2099,12 +2110,14 @@
         <v>58</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="6"/>
+        <v>99</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>97</v>
+      </c>
       <c r="D2" t="str">
         <f>"sc create "&amp;B2&amp;" binPath= """&amp;B3&amp;""" start= auto"</f>
-        <v>sc create ServiceOCR1 binPath= "C:\SourceWeb\SERVICE\ServiceOCR\DocProService.exe" start= auto</v>
+        <v>sc create ServiceOCR11 binPath= "C:\SourceWeb\SERVICE\ServiceOCR\DocProService.exe" start= auto</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2123,7 +2136,9 @@
       <c r="B4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="6"/>
+      <c r="C4" s="6" t="s">
+        <v>98</v>
+      </c>
       <c r="D4" t="str">
         <f>"sc create "&amp;B4&amp;" binPath= """&amp;B5&amp;""" start= auto"</f>
         <v>sc create ServiceExport binPath= "C:\SourceWeb\SERVICE\ServiceExport\DocProService.exe" start= auto</v>
@@ -2150,7 +2165,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1500CE9D-A3F9-42DA-B277-1145613BDD26}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -2158,24 +2173,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="49" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="33" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="B2" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="B2" s="49" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="50" t="s">
-        <v>85</v>
+      <c r="A3" s="35" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -2215,16 +2230,16 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="51" t="s">
+      <c r="A10" s="36" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="34" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="48" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="49" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -2234,21 +2249,21 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="51" t="s">
-        <v>91</v>
+      <c r="A13" s="36" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>93</v>
-      </c>
-      <c r="B14" s="49" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="52" t="s">
-        <v>94</v>
       </c>
       <c r="B15" t="str">
         <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;""" /&gt;"</f>
@@ -2256,8 +2271,8 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="52" t="s">
-        <v>95</v>
+      <c r="A16" t="s">
+        <v>94</v>
       </c>
       <c r="B16" t="str">
         <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;"\Storage\Files"" /&gt;"</f>
@@ -2265,12 +2280,22 @@
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="52" t="s">
-        <v>96</v>
+      <c r="A17" t="s">
+        <v>95</v>
       </c>
       <c r="B17" t="str">
         <f>"&lt;add key=""StgDir"" value="""&amp;$B$14&amp;""" /&gt;"</f>
         <v>&lt;add key="StgDir" value="C:\AXE\DataStorage" /&gt;</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2279,6 +2304,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010097FE9C0C8E574444875F1CBBF8414DDA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c7e0992f45b677c2156c5ab52d17057f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="97d068c0-5bfb-413b-9996-819e39fdf128" xmlns:ns3="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f06a3ea3329379ac3c4a4f5da7fed49" ns2:_="" ns3:_="">
     <xsd:import namespace="97d068c0-5bfb-413b-9996-819e39fdf128"/>
@@ -2513,28 +2559,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
+    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
-    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E3A15DF-6B1B-40AC-992D-CB264AF46DCF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2551,23 +2595,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
-    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>